<commit_message>
Refresh Skybase September DR and true-ups from settle-dr-dune main
</commit_message>
<xml_diff>
--- a/settlements/skybase/2026-09/skybase_settlement_september_2026.xlsx
+++ b/settlements/skybase/2026-09/skybase_settlement_september_2026.xlsx
@@ -7,12 +7,11 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Close status" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Venues" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Sky Revenue" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Sky Direct" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Debt" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Venues" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Sky Revenue" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Sky Direct" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Debt" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -77,7 +76,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -93,12 +92,6 @@
     <xf numFmtId="167" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -464,144 +457,6 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B10"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="42" customWidth="1" min="1" max="1"/>
-    <col width="115" customWidth="1" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="13" t="inlineStr">
-        <is>
-          <t>September 2026 close</t>
-        </is>
-      </c>
-      <c r="B1" s="13" t="inlineStr">
-        <is>
-          <t>Official reference-rate coverage complete</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="14" t="inlineStr">
-        <is>
-          <t>calculation</t>
-        </is>
-      </c>
-      <c r="B2" s="14" t="inlineStr">
-        <is>
-          <t>Independent full monthly pipeline, compared field-by-field with September 30 API result</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="14" t="inlineStr">
-        <is>
-          <t>calculation_code_version</t>
-        </is>
-      </c>
-      <c r="B3" s="14" t="inlineStr">
-        <is>
-          <t>c32f25a7ef410eaaf9212b8f546f652c715dc7ac</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="14" t="inlineStr">
-        <is>
-          <t>daily_revision</t>
-        </is>
-      </c>
-      <c r="B4" s="14" t="inlineStr">
-        <is>
-          <t>9824ec82a2122e4ab9d1b521c89e7c2b08cfce4fd36c574ff8ca27779f851fd3</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="14" t="inlineStr">
-        <is>
-          <t>monthly_result_sha256</t>
-        </is>
-      </c>
-      <c r="B5" s="14" t="inlineStr">
-        <is>
-          <t>634e859964fa60ea684f5a77f894ed8dc24990c72da7339922d096b6005aa94a</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="14" t="inlineStr">
-        <is>
-          <t>daily_result_sha256</t>
-        </is>
-      </c>
-      <c r="B6" s="14" t="inlineStr">
-        <is>
-          <t>634e859964fa60ea684f5a77f894ed8dc24990c72da7339922d096b6005aa94a</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="14" t="inlineStr">
-        <is>
-          <t>comparison</t>
-        </is>
-      </c>
-      <c r="B7" s="14" t="inlineStr">
-        <is>
-          <t>all result fields match</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="14" t="inlineStr">
-        <is>
-          <t>distribution_rewards_workbook_sha256</t>
-        </is>
-      </c>
-      <c r="B8" s="14" t="inlineStr">
-        <is>
-          <t>17eee2ca39bd63e68e6d87097ede0007d8741e41cb9a7fceb017da713103b02e</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="14" t="inlineStr">
-        <is>
-          <t>distribution_rewards_code</t>
-        </is>
-      </c>
-      <c r="B9" s="14" t="inlineStr">
-        <is>
-          <t>1e9ecb2 (merged settle-dr-dune PR #27; finalized September snapshot)</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="14" t="inlineStr">
-        <is>
-          <t>reference_rate_status</t>
-        </is>
-      </c>
-      <c r="B10" s="14" t="inlineStr">
-        <is>
-          <t>official coverage complete</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
   <dimension ref="A1:B31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -655,12 +510,13 @@
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>106035.3530694837</v>
+        <v>105735.7496915168</v>
       </c>
     </row>
     <row r="7">
+      <c r="A7" t="inlineStr"/>
       <c r="B7" s="4" t="n">
-        <v>144111.3589897424</v>
+        <v>143811.7556117754</v>
       </c>
     </row>
     <row r="9">
@@ -696,6 +552,7 @@
       </c>
     </row>
     <row r="12">
+      <c r="A12" t="inlineStr"/>
       <c r="B12" s="4" t="n">
         <v>0</v>
       </c>
@@ -733,6 +590,7 @@
       </c>
     </row>
     <row r="17">
+      <c r="A17" t="inlineStr"/>
       <c r="B17" s="4" t="n">
         <v>0</v>
       </c>
@@ -756,7 +614,7 @@
         </is>
       </c>
       <c r="B20" s="5" t="n">
-        <v>144111.3589897424</v>
+        <v>143811.7556117754</v>
       </c>
     </row>
     <row r="21">
@@ -766,7 +624,7 @@
         </is>
       </c>
       <c r="B21" s="5" t="n">
-        <v>27740.235315</v>
+        <v>41560.042993</v>
       </c>
     </row>
     <row r="22">
@@ -776,7 +634,7 @@
         </is>
       </c>
       <c r="B22" s="5" t="n">
-        <v>34229.172646</v>
+        <v>71804.679106</v>
       </c>
     </row>
     <row r="23">
@@ -786,7 +644,7 @@
         </is>
       </c>
       <c r="B23" s="5" t="n">
-        <v>758.752668</v>
+        <v>1782.888077</v>
       </c>
     </row>
     <row r="24">
@@ -800,8 +658,9 @@
       </c>
     </row>
     <row r="25">
+      <c r="A25" t="inlineStr"/>
       <c r="B25" s="6" t="n">
-        <v>268805.6895307424</v>
+        <v>320925.5356997754</v>
       </c>
     </row>
     <row r="26">
@@ -843,7 +702,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2026-10-01T10:53:32+00:00</t>
+          <t>2026-10-01T15:36:11+00:00</t>
         </is>
       </c>
     </row>
@@ -864,7 +723,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -996,7 +855,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1077,7 +936,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1162,7 +1021,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2466,6 +2325,15 @@
           <t>Σ daily charges</t>
         </is>
       </c>
+      <c r="B37" t="inlineStr"/>
+      <c r="C37" t="inlineStr"/>
+      <c r="D37" t="inlineStr"/>
+      <c r="E37" t="inlineStr"/>
+      <c r="F37" t="inlineStr"/>
+      <c r="G37" t="inlineStr"/>
+      <c r="H37" t="inlineStr"/>
+      <c r="I37" t="inlineStr"/>
+      <c r="J37" t="inlineStr"/>
       <c r="K37" s="12" t="n">
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
Refresh Skybase September DR, true-ups and downstream reports (#224)
</commit_message>
<xml_diff>
--- a/settlements/skybase/2026-09/skybase_settlement_september_2026.xlsx
+++ b/settlements/skybase/2026-09/skybase_settlement_september_2026.xlsx
@@ -7,12 +7,11 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Close status" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Venues" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Sky Revenue" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Sky Direct" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Debt" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Venues" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Sky Revenue" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Sky Direct" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Debt" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -77,7 +76,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -93,12 +92,6 @@
     <xf numFmtId="167" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -464,144 +457,6 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B10"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="42" customWidth="1" min="1" max="1"/>
-    <col width="115" customWidth="1" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="13" t="inlineStr">
-        <is>
-          <t>September 2026 close</t>
-        </is>
-      </c>
-      <c r="B1" s="13" t="inlineStr">
-        <is>
-          <t>Official reference-rate coverage complete</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="14" t="inlineStr">
-        <is>
-          <t>calculation</t>
-        </is>
-      </c>
-      <c r="B2" s="14" t="inlineStr">
-        <is>
-          <t>Independent full monthly pipeline, compared field-by-field with September 30 API result</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="14" t="inlineStr">
-        <is>
-          <t>calculation_code_version</t>
-        </is>
-      </c>
-      <c r="B3" s="14" t="inlineStr">
-        <is>
-          <t>c32f25a7ef410eaaf9212b8f546f652c715dc7ac</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="14" t="inlineStr">
-        <is>
-          <t>daily_revision</t>
-        </is>
-      </c>
-      <c r="B4" s="14" t="inlineStr">
-        <is>
-          <t>9824ec82a2122e4ab9d1b521c89e7c2b08cfce4fd36c574ff8ca27779f851fd3</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="14" t="inlineStr">
-        <is>
-          <t>monthly_result_sha256</t>
-        </is>
-      </c>
-      <c r="B5" s="14" t="inlineStr">
-        <is>
-          <t>634e859964fa60ea684f5a77f894ed8dc24990c72da7339922d096b6005aa94a</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="14" t="inlineStr">
-        <is>
-          <t>daily_result_sha256</t>
-        </is>
-      </c>
-      <c r="B6" s="14" t="inlineStr">
-        <is>
-          <t>634e859964fa60ea684f5a77f894ed8dc24990c72da7339922d096b6005aa94a</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="14" t="inlineStr">
-        <is>
-          <t>comparison</t>
-        </is>
-      </c>
-      <c r="B7" s="14" t="inlineStr">
-        <is>
-          <t>all result fields match</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="14" t="inlineStr">
-        <is>
-          <t>distribution_rewards_workbook_sha256</t>
-        </is>
-      </c>
-      <c r="B8" s="14" t="inlineStr">
-        <is>
-          <t>17eee2ca39bd63e68e6d87097ede0007d8741e41cb9a7fceb017da713103b02e</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="14" t="inlineStr">
-        <is>
-          <t>distribution_rewards_code</t>
-        </is>
-      </c>
-      <c r="B9" s="14" t="inlineStr">
-        <is>
-          <t>1e9ecb2 (merged settle-dr-dune PR #27; finalized September snapshot)</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="14" t="inlineStr">
-        <is>
-          <t>reference_rate_status</t>
-        </is>
-      </c>
-      <c r="B10" s="14" t="inlineStr">
-        <is>
-          <t>official coverage complete</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
   <dimension ref="A1:B31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -655,12 +510,13 @@
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>106035.3530694837</v>
+        <v>105735.7496915168</v>
       </c>
     </row>
     <row r="7">
+      <c r="A7" t="inlineStr"/>
       <c r="B7" s="4" t="n">
-        <v>144111.3589897424</v>
+        <v>143811.7556117754</v>
       </c>
     </row>
     <row r="9">
@@ -696,6 +552,7 @@
       </c>
     </row>
     <row r="12">
+      <c r="A12" t="inlineStr"/>
       <c r="B12" s="4" t="n">
         <v>0</v>
       </c>
@@ -733,6 +590,7 @@
       </c>
     </row>
     <row r="17">
+      <c r="A17" t="inlineStr"/>
       <c r="B17" s="4" t="n">
         <v>0</v>
       </c>
@@ -756,7 +614,7 @@
         </is>
       </c>
       <c r="B20" s="5" t="n">
-        <v>144111.3589897424</v>
+        <v>143811.7556117754</v>
       </c>
     </row>
     <row r="21">
@@ -766,7 +624,7 @@
         </is>
       </c>
       <c r="B21" s="5" t="n">
-        <v>27740.235315</v>
+        <v>41560.042993</v>
       </c>
     </row>
     <row r="22">
@@ -776,7 +634,7 @@
         </is>
       </c>
       <c r="B22" s="5" t="n">
-        <v>34229.172646</v>
+        <v>71804.679106</v>
       </c>
     </row>
     <row r="23">
@@ -786,7 +644,7 @@
         </is>
       </c>
       <c r="B23" s="5" t="n">
-        <v>758.752668</v>
+        <v>1782.888077</v>
       </c>
     </row>
     <row r="24">
@@ -800,8 +658,9 @@
       </c>
     </row>
     <row r="25">
+      <c r="A25" t="inlineStr"/>
       <c r="B25" s="6" t="n">
-        <v>268805.6895307424</v>
+        <v>320925.5356997754</v>
       </c>
     </row>
     <row r="26">
@@ -843,7 +702,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2026-10-01T10:53:32+00:00</t>
+          <t>2026-10-01T15:36:11+00:00</t>
         </is>
       </c>
     </row>
@@ -864,7 +723,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -996,7 +855,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1077,7 +936,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1162,7 +1021,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2466,6 +2325,15 @@
           <t>Σ daily charges</t>
         </is>
       </c>
+      <c r="B37" t="inlineStr"/>
+      <c r="C37" t="inlineStr"/>
+      <c r="D37" t="inlineStr"/>
+      <c r="E37" t="inlineStr"/>
+      <c r="F37" t="inlineStr"/>
+      <c r="G37" t="inlineStr"/>
+      <c r="H37" t="inlineStr"/>
+      <c r="I37" t="inlineStr"/>
+      <c r="J37" t="inlineStr"/>
       <c r="K37" s="12" t="n">
         <v>0</v>
       </c>

</xml_diff>